<commit_message>
Usun polaczenie SQL z makra VBA generatora planu pracy - przenies do PowerShell
Makro Excela (modGeneratorPlanuPracy.bas) nie moze laczyc sie z baza SQL
(wymog bezpieczenstwa klienta). Generator dzieli sie teraz na dwa kroki:
makro generuje XML z placeholderem guid="KOD:<Kod pracownika>" bez zadnego
polaczenia z SQL, a nowy skrypt Importuj-PlanyPracy.ps1 (uruchamiany poza
Excelem) rozwiazuje placeholder na prawdziwy GUID kalendarza indywidualnego
pracownika (bez znaczenia jaki kalendarz ma pracownik) i wywoluje dbmgr
importxml.

Ustalono empirycznie (proby na bazie Claude), ze KalendarzBase nie ma
zadnego pola uzytecznego w where/key poza Guid - udokumentowane w
Generator planu pracy.md. Pelny pipeline (placeholder -> PowerShell ->
dbmgr) zweryfikowany na zywo dla pracownika PP-01.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QfvTh9rkSZxCKcn3RD5j2v
</commit_message>
<xml_diff>
--- a/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
+++ b/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
@@ -27,10 +27,10 @@
     <t>Generator cyklicznego importu planu pracy (dnia planu) do enova365</t>
   </si>
   <si>
-    <t>Ten skoroszyt + makro VBA generuja pliki XML importu „dnia planu” (zakladka Kalendarz / Norma czasu pracy w kartotece pracownika, tabela DniKalendarza, wiersze typu Soneta.Kalend.DzienPlanu) na podstawie danych wpisanych w arkuszu „Plan”. Wygenerowane pliki importuje sie standardowo poleceniem dbmgr importxml &lt;baza&gt; "&lt;plik&gt;" w trybie standard.</t>
-  </si>
-  <si>
-    <t>1. Uzupelnij arkusz „Konfiguracja”: adres serwera SQL i nazwa bazy enova (Windows Auth), folder docelowy na pliki XML oraz GUID-y definicji dnia/strefy (domyslne pasuja do standardowej konfiguracji enova365 i zwykle nie trzeba ich zmieniac).</t>
+    <t>Ten skoroszyt + makro VBA generuja pliki XML importu „dnia planu” (zakladka Kalendarz / Norma czasu pracy w kartotece pracownika, tabela DniKalendarza, wiersze typu Soneta.Kalend.DzienPlanu) na podstawie danych wpisanych w arkuszu „Plan”. WAZNE: makro VBA NIE LACZY SIE Z BAZA SQL (zakaz polaczen z Excela) - generuje pliki z placeholderem zamiast GUID-u kalendarza. Dokonczenie (rozwiazanie placeholdera + import) robi OSOBNY skrypt PowerShell Importuj-PlanyPracy.ps1, uruchamiany POZA Excelem.</t>
+  </si>
+  <si>
+    <t>1. Uzupelnij arkusz „Konfiguracja”: folder docelowy na pliki XML, GUID-y definicji dnia/strefy (domyslne pasuja do standardowej konfiguracji enova365) oraz SQL Server/Baza (potrzebne dopiero w kroku 6, dla skryptu PowerShell - nie dla makra).</t>
   </si>
   <si>
     <t>2. Uzupelnij arkusz „Plan” - jeden wiersz = jeden zakres dat dla jednego pracownika. Kolumny Pn..Nd: wpisz dowolny znak (np. X) w dniach tygodnia, ktore maja byc dniami pracy wg podanych stref. Kolumny Strefa 1..4: godzina rozpoczecia i czas trwania kazdej strefy (format G:MM albo komorka sformatowana jako Godzina), np. Strefa 1 = 8:00 / 4:00, Strefa 2 = 13:00 / 4:00 (przerwa 12:00-13:00 wynika sama z luki miedzy strefami - nie wpisuje sie jej).</t>
@@ -39,16 +39,16 @@
     <t>3. W Excelu: Alt+F11 (Edytor VBA) -&gt; Plik -&gt; Importuj plik... -&gt; wskaz modGeneratorPlanuPracy.bas (w tym samym folderze co ten skoroszyt). Zapisz skoroszyt jako .xlsm (Excel z obsluga makr).</t>
   </si>
   <si>
-    <t>4. Uruchom makro GenerujPlanyPracy (Alt+F8 -&gt; GenerujPlanyPracy -&gt; Uruchom), albo przypisz je do przycisku na arkuszu „Plan” (Deweloper -&gt; Wstaw -&gt; Przycisk).</t>
-  </si>
-  <si>
-    <t>5. Makro laczy sie z baza SQL, dla kazdego Kodu pracownika odczytuje GUID jego indywidualnego kalendarza (Kalendarze.Typ=2), rozwija zakresy dat na konkretne dni wedlug zaznaczonych dni tygodnia i zapisuje po jednym pliku XML na pracownika w folderze docelowym.</t>
-  </si>
-  <si>
-    <t>6. WAZNE: pracownik musi juz istniec w enova z zapisanym Etatem (indywidualny kalendarz powstaje automatycznie przy zapisie Etat) - inaczej makro zglosi blad braku kalendarza dla danego Kodu.</t>
-  </si>
-  <si>
-    <t>7. WAZNE: fromto w wygenerowanym pliku obejmuje caly zakres od najwczesniejszej do najpozniejszej wygenerowanej daty dla danego pracownika. Ponowny import ZASTEPUJE cala zawartosc dni planu w tym zakresie - jesli w danym okresie sa dni robocze celowo pominiete w arkuszu (np. planowana nieobecnosc), trzeba je swiadomie uwzglednic, inaczez przy reimporcie wroca do planu domyslnego z kalendarza wzorcowego.</t>
+    <t>4. Uruchom makro GenerujPlanyPracy (Alt+F8 -&gt; GenerujPlanyPracy -&gt; Uruchom), albo przypisz je do przycisku na arkuszu „Plan” (Deweloper -&gt; Wstaw -&gt; Przycisk). Makro NIE LACZY SIE Z SQL - rozwija zakresy dat na konkretne dni wedlug zaznaczonych dni tygodnia i zapisuje po jednym pliku XML na pracownika w folderze docelowym, z placeholderem guid="KOD:&lt;Kod pracownika&gt;" zamiast prawdziwego GUID-u kalendarza.</t>
+  </si>
+  <si>
+    <t>5. WAZNE: pracownik musi juz istniec w enova z zapisanym Etatem (jego indywidualny kalendarz powstaje wtedy automatycznie) - inaczej krok 6 zglosi blad braku kalendarza dla danego Kodu i POMINIE caly plik tego pracownika (reszta plikow zaimportuje sie normalnie).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. POZA Excelem uruchom (PowerShell): .\Importuj-PlanyPracy.ps1 -SqlServer „...” -Baza „...” -Importuj  - ten skrypt laczy sie z SQL (Windows Auth), podmienia placeholder na prawdziwy GUID kalendarza indywidualnego (Kalendarze.Typ=2, bez znaczenia jaki konkretnie kalendarz ma pracownik) i wywoluje dbmgr importxml. Bez przelacznika -Importuj tylko przygotowuje pliki *.gotowy.xml do recznego zaimportowania.</t>
+  </si>
+  <si>
+    <t>7. WAZNE: fromto w wygenerowanym pliku obejmuje caly zakres od najwczesniejszej do najpozniejszej wygenerowanej daty dla danego pracownika. Ponowny import ZASTEPUJE cala zawartosc dni planu w tym zakresie - jesli w danym okresie sa dni robocze celowo pominiete w arkuszu (np. planowana nieobecnosc), trzeba je swiadomie uwzglednic, inaczej przy reimporcie wroca do planu domyslnego z kalendarza wzorcowego.</t>
   </si>
   <si>
     <t>8. Zawsze najpierw testowac wygenerowany plik na bazie testowej, dopiero potem na produkcyjnej.</t>
@@ -63,7 +63,7 @@
     <t>localhost\SQLEXPRESS</t>
   </si>
   <si>
-    <t>Adres serwera SQL bazy enova (jak w polaczeniu Windows Auth).</t>
+    <t>NIE jest czytane przez makro (makro nie laczy sie z SQL) - to tylko notatka, jakiej wartosci -SqlServer uzyc przy uruchamianiu Importuj-PlanyPracy.ps1 w kroku 6.</t>
   </si>
   <si>
     <t>Baza danych</t>
@@ -72,7 +72,7 @@
     <t>Claude</t>
   </si>
   <si>
-    <t>Nazwa bazy enova, do ktorej trafia import (np. Claude = baza testowa).</t>
+    <t>NIE jest czytane przez makro - notatka do parametru -Baza skryptu Importuj-PlanyPracy.ps1 (krok 6).</t>
   </si>
   <si>
     <t>Folder na pliki XML</t>
@@ -81,7 +81,7 @@
     <t>C:\enovaServer\Projekty\Enova\ImportyXML\</t>
   </si>
   <si>
-    <t>Folder docelowy na wygenerowane pliki (ze slashem na koncu).</t>
+    <t>Folder docelowy na wygenerowane pliki (ze slashem na koncu) - czyta je makro.</t>
   </si>
   <si>
     <t>GUID: Definicja dnia „Pracy”</t>

</xml_diff>

<commit_message>
Napraw domyslny folder docelowy w generatorze planu pracy
Domyslna sciezka w Konfiguracji ("C:\enovaServer\Projekty\Enova\ImportyXML\")
byla ze srodowiska deweloperskiego i nie istnieje na komputerze
uzytkownika - powodowalo to cichy blad zapisu, bez widocznego pliku
wynikowego. Puste pole oznacza teraz zapis obok samego skoroszytu,
tworzenie folderu obsluguje wiele brakujacych poziomow naraz, a bledy
folderu/zapisu pokazuja czytelny komunikat zamiast cichego niepowodzenia.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QfvTh9rkSZxCKcn3RD5j2v
</commit_message>
<xml_diff>
--- a/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
+++ b/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
@@ -30,7 +30,7 @@
     <t>Ten skoroszyt + makro VBA generuja plik XML w OFICJALNYM formacie enova (Root/DniPlanu/DzienPlanu/Strefy - ten sam format co wzorcowy arkusz Soneta „xml- Norma pracy.xlsm”) na podstawie danych wpisanych w arkuszu „Plan”. Makro NIE LACZY SIE Z BAZA SQL W OGOLE - pracownik jest identyfikowany WYLACZNIE po kodzie (&lt;Pracownik&gt;), a importer enova sam go wyszukuje. Gotowy plik importuje sie w programie enova: Plik | Importuj zapisy | Import czasu pracy i wynagrodzen.</t>
   </si>
   <si>
-    <t>1. Uzupelnij arkusz „Konfiguracja”: folder docelowy na plik XML oraz nazwy definicji dnia/strefy (domyslnie „Pracy” / „Praca w normie” - standardowe nazwy w enova365; zmien tylko jesli w Twojej bazie maja inne nazwy).</t>
+    <t>1. Arkusz „Konfiguracja”: pole „Folder na plik XML” zostaw PUSTE (plik zapisze sie obok tego skoroszytu) - chyba ze chcesz wskazac inny, JUZ ISTNIEJACY na Twoim komputerze folder. Nazwy definicji dnia/strefy zmien tylko jesli w Twojej bazie enova roznia sie od domyslnych „Pracy” / „Praca w normie”.</t>
   </si>
   <si>
     <t>2. Uzupelnij arkusz „Plan” - jeden wiersz = jeden zakres dat dla jednego pracownika (Kod pracownika - dokladnie taki jak w kartotece enova). Kolumny Pn..Nd: wpisz dowolny znak (np. X) w dniach tygodnia, ktore maja byc dniami pracy wg podanych stref. Kolumny Strefa 1..4: godzina rozpoczecia i czas trwania kazdej strefy (format G:MM albo komorka sformatowana jako Godzina), np. Strefa 1 = 8:00 / 4:00, Strefa 2 = 13:00 / 4:00 (przerwa 12:00-13:00 wynika sama z luki miedzy strefami - nie wpisuje sie jej).</t>
@@ -60,10 +60,10 @@
     <t>Folder na plik XML</t>
   </si>
   <si>
-    <t>C:\enovaServer\Projekty\Enova\ImportyXML\</t>
-  </si>
-  <si>
-    <t>Folder docelowy na wygenerowany plik (ze slashem na koncu).</t>
+    <t/>
+  </si>
+  <si>
+    <t>PUSTE (zalecane) = plik zapisze sie w tym samym folderze co ten skoroszyt. Mozesz wpisac inny istniejacy folder (np. C:\Migracja\, jak w oryginalnym arkuszu Soneta) - musi juz istniec na TWOIM komputerze, inaczej makro zglosi blad.</t>
   </si>
   <si>
     <t>Nazwa definicji dnia</t>
@@ -154,9 +154,6 @@
   </si>
   <si>
     <t>X</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>8:00</t>
@@ -845,37 +842,37 @@
         <v>43</v>
       </c>
       <c r="I2" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" t="s">
+        <v>12</v>
+      </c>
+      <c r="K2" t="s">
         <v>44</v>
       </c>
-      <c r="J2" t="s">
-        <v>44</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>45</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>46</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
+        <v>45</v>
+      </c>
+      <c r="O2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>12</v>
+      </c>
+      <c r="R2" t="s">
+        <v>12</v>
+      </c>
+      <c r="S2" t="s">
         <v>47</v>
-      </c>
-      <c r="N2" t="s">
-        <v>46</v>
-      </c>
-      <c r="O2" t="s">
-        <v>44</v>
-      </c>
-      <c r="P2" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>44</v>
-      </c>
-      <c r="R2" t="s">
-        <v>44</v>
-      </c>
-      <c r="S2" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Generator planu pracy: uproszcz arkusz Plan do jednego wiersza na dzien
Wg wzorcowego pliku Excela dostarczonego przez uzytkownika - usuniete
kolumny Data do / Pn..Nd, kazdy wiersz to teraz jeden konkretny dzien
jednego pracownika. Makro juz nie rozwija zakresow dat/dni tygodnia.
Nadal zero SQL, zero GUID.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AiyfQjJpMAiDQoFVsuEyaK
</commit_message>
<xml_diff>
--- a/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
+++ b/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Plan" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Plan!$A$1:$S$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Plan!$A$1:$J$12</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -33,13 +33,13 @@
     <t>1. Arkusz „Konfiguracja”: pole „Folder na plik XML” zostaw PUSTE (plik zapisze sie obok tego skoroszytu) - chyba ze chcesz wskazac inny, JUZ ISTNIEJACY na Twoim komputerze folder. Nazwy definicji dnia/strefy zmien tylko jesli w Twojej bazie enova roznia sie od domyslnych „Pracy” / „Praca w normie”.</t>
   </si>
   <si>
-    <t>2. Uzupelnij arkusz „Plan” - jeden wiersz = jeden zakres dat dla jednego pracownika (Kod pracownika - dokladnie taki jak w kartotece enova). Kolumny Pn..Nd: wpisz dowolny znak (np. X) w dniach tygodnia, ktore maja byc dniami pracy wg podanych stref. Kolumny Strefa 1..4: godzina rozpoczecia i czas trwania kazdej strefy (format G:MM albo komorka sformatowana jako Godzina), np. Strefa 1 = 8:00 / 4:00, Strefa 2 = 13:00 / 4:00 (przerwa 12:00-13:00 wynika sama z luki miedzy strefami - nie wpisuje sie jej).</t>
+    <t>2. Uzupelnij arkusz „Plan” - jeden wiersz = jeden dzien dla jednego pracownika (Kod pracownika - dokladnie taki jak w kartotece enova - oraz Data tego konkretnego dnia). Zadnego zakresu dat ani zaznaczania dni tygodnia - jesli pracownik ma pracowac np. caly wrzesien od poniedzialku do piatku, kazdy z tych dni to OSOBNY wiersz w arkuszu. Kolumny Strefa 1..4: godzina rozpoczecia i czas trwania kazdej strefy tego dnia (format G:MM albo komorka sformatowana jako Godzina), np. Strefa 1 = 8:00 / 4:00, Strefa 2 = 13:00 / 4:00 (przerwa 12:00-13:00 wynika sama z luki miedzy strefami - nie wpisuje sie jej). Dzien z jedna strefa - wypelnij tylko Strefa 1, reszte zostaw pusta.</t>
   </si>
   <si>
     <t>3. W Excelu: Alt+F11 (Edytor VBA) -&gt; Plik -&gt; Importuj plik... -&gt; wskaz modGeneratorPlanuPracy.bas (w tym samym folderze co ten skoroszyt). Zapisz skoroszyt jako .xlsm (Excel z obsluga makr).</t>
   </si>
   <si>
-    <t>4. Uruchom makro GenerujPlanyPracy (Alt+F8 -&gt; GenerujPlanyPracy -&gt; Uruchom), albo przypisz je do przycisku na arkuszu „Plan” (Deweloper -&gt; Wstaw -&gt; Przycisk). Makro NIE LACZY SIE Z SQL W OGOLE - rozwija zakresy dat na konkretne dni wedlug zaznaczonych dni tygodnia i zapisuje JEDEN plik XML (wszyscy pracownicy z arkusza razem) w formacie Root/DniPlanu/DzienPlanu/Strefy, identyfikujac kazdy dzien wylacznie po kodzie pracownika.</t>
+    <t>4. Uruchom makro GenerujPlanyPracy (Alt+F8 -&gt; GenerujPlanyPracy -&gt; Uruchom), albo przypisz je do przycisku na arkuszu „Plan” (Deweloper -&gt; Wstaw -&gt; Przycisk). Makro NIE LACZY SIE Z SQL W OGOLE - dla kazdego wiersza arkusza zapisuje jeden dzien planu, wszystkie wiersze/pracownikow razem w JEDNYM pliku XML w formacie Root/DniPlanu/DzienPlanu/Strefy, identyfikujac kazdy dzien wylacznie po kodzie pracownika.</t>
   </si>
   <si>
     <t>5. Zaimportuj gotowy plik w programie enova: Plik | Importuj zapisy | Import czasu pracy i wynagrodzen (wymaga zarejestrowanego w docelowej bazie rozszerzenia Soneta.CzasPracy.Migrator/Soneta.CzasPracy.Utils - bez tego pozycja menu jest niewidoczna).</t>
@@ -96,31 +96,7 @@
     <t>Kod pracownika</t>
   </si>
   <si>
-    <t>Data od</t>
-  </si>
-  <si>
-    <t>Data do</t>
-  </si>
-  <si>
-    <t>Pn</t>
-  </si>
-  <si>
-    <t>Wt</t>
-  </si>
-  <si>
-    <t>Śr</t>
-  </si>
-  <si>
-    <t>Czw</t>
-  </si>
-  <si>
-    <t>Pt</t>
-  </si>
-  <si>
-    <t>Sob</t>
-  </si>
-  <si>
-    <t>Nd</t>
+    <t>Data</t>
   </si>
   <si>
     <t>Strefa 1 od</t>
@@ -147,15 +123,9 @@
     <t>Strefa 4 czas</t>
   </si>
   <si>
-    <t>Uwagi</t>
-  </si>
-  <si>
     <t>PP-01</t>
   </si>
   <si>
-    <t>X</t>
-  </si>
-  <si>
     <t>8:00</t>
   </si>
   <si>
@@ -163,9 +133,6 @@
   </si>
   <si>
     <t>13:00</t>
-  </si>
-  <si>
-    <t>Przyklad - patrz plik testowy ImportyXML\Generator planu pracy\Norma pracy - test PP-01 2026-11-05 dwie strefy.xml</t>
   </si>
 </sst>
 </file>
@@ -738,23 +705,14 @@
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="5.7109375" customWidth="1"/>
-    <col min="5" max="5" width="5.7109375" customWidth="1"/>
-    <col min="6" max="6" width="5.7109375" customWidth="1"/>
-    <col min="7" max="7" width="5.7109375" customWidth="1"/>
-    <col min="8" max="8" width="5.7109375" customWidth="1"/>
-    <col min="9" max="9" width="5.7109375" customWidth="1"/>
-    <col min="10" max="10" width="5.7109375" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.7109375" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" customWidth="1"/>
-    <col min="14" max="14" width="12.7109375" customWidth="1"/>
-    <col min="15" max="15" width="11.7109375" customWidth="1"/>
-    <col min="16" max="16" width="12.7109375" customWidth="1"/>
-    <col min="17" max="17" width="11.7109375" customWidth="1"/>
-    <col min="18" max="18" width="12.7109375" customWidth="1"/>
-    <col min="19" max="19" width="55.710938" customWidth="1"/>
+    <col min="3" max="3" width="11.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="7.2" customHeight="1">
@@ -788,94 +746,228 @@
       <c r="J1" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="K1" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q1" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="R1" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="S1" s="8" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B2" s="9">
         <v>46266</v>
       </c>
-      <c r="C2" s="9">
-        <v>46295</v>
+      <c r="C2" t="s">
+        <v>34</v>
       </c>
       <c r="D2" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="E2" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>43</v>
-      </c>
-      <c r="G2" t="s">
-        <v>43</v>
-      </c>
-      <c r="H2" t="s">
-        <v>43</v>
-      </c>
-      <c r="I2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" t="s">
-        <v>44</v>
-      </c>
-      <c r="L2" t="s">
-        <v>45</v>
-      </c>
-      <c r="M2" t="s">
-        <v>46</v>
-      </c>
-      <c r="N2" t="s">
-        <v>45</v>
-      </c>
-      <c r="O2" t="s">
-        <v>12</v>
-      </c>
-      <c r="P2" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>12</v>
-      </c>
-      <c r="R2" t="s">
-        <v>12</v>
-      </c>
-      <c r="S2" t="s">
-        <v>47</v>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="9">
+        <v>46267</v>
+      </c>
+      <c r="C3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="9">
+        <v>46268</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="9">
+        <v>46269</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="9">
+        <v>46270</v>
+      </c>
+      <c r="C6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="9">
+        <v>46271</v>
+      </c>
+      <c r="C7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="9">
+        <v>46272</v>
+      </c>
+      <c r="C8" t="s">
+        <v>34</v>
+      </c>
+      <c r="D8" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="9">
+        <v>46273</v>
+      </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="9">
+        <v>46274</v>
+      </c>
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D10" t="s">
+        <v>35</v>
+      </c>
+      <c r="E10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="9">
+        <v>46275</v>
+      </c>
+      <c r="C11" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" t="s">
+        <v>35</v>
+      </c>
+      <c r="E11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="9">
+        <v>46276</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S2"/>
+  <autoFilter ref="A1:J12"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Generator planu pracy: dodaj kolumne Nazwa dnia (napraw pusta Definicje)
Realny test importu zglosil "Definicja dnia o nazwie '' nie zostala
znaleziona" - Definicja brana byla wylacznie z globalnej Konfiguracja,
ktora wyszla pusta. Arkusz Plan ma teraz kolumne C "Nazwa dnia" per
wiersz (fallback na Konfiguracja!B3 gdy pusta, blad gdy oba puste).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AiyfQjJpMAiDQoFVsuEyaK
</commit_message>
<xml_diff>
--- a/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
+++ b/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Plan" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Plan!$A$1:$J$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Plan!$A$1:$K$12</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -33,7 +33,7 @@
     <t>1. Arkusz „Konfiguracja”: pole „Folder na plik XML” zostaw PUSTE (plik zapisze sie obok tego skoroszytu) - chyba ze chcesz wskazac inny, JUZ ISTNIEJACY na Twoim komputerze folder. Nazwy definicji dnia/strefy zmien tylko jesli w Twojej bazie enova roznia sie od domyslnych „Pracy” / „Praca w normie”.</t>
   </si>
   <si>
-    <t>2. Uzupelnij arkusz „Plan” - jeden wiersz = jeden dzien dla jednego pracownika (Kod pracownika - dokladnie taki jak w kartotece enova - oraz Data tego konkretnego dnia). Zadnego zakresu dat ani zaznaczania dni tygodnia - jesli pracownik ma pracowac np. caly wrzesien od poniedzialku do piatku, kazdy z tych dni to OSOBNY wiersz w arkuszu. Kolumny Strefa 1..4: godzina rozpoczecia i czas trwania kazdej strefy tego dnia (format G:MM albo komorka sformatowana jako Godzina), np. Strefa 1 = 8:00 / 4:00, Strefa 2 = 13:00 / 4:00 (przerwa 12:00-13:00 wynika sama z luki miedzy strefami - nie wpisuje sie jej). Dzien z jedna strefa - wypelnij tylko Strefa 1, reszte zostaw pusta.</t>
+    <t>2. Uzupelnij arkusz „Plan” - jeden wiersz = jeden dzien dla jednego pracownika (Kod pracownika - dokladnie taki jak w kartotece enova - oraz Data tego konkretnego dnia). Zadnego zakresu dat ani zaznaczania dni tygodnia - jesli pracownik ma pracowac np. caly wrzesien od poniedzialku do piatku, kazdy z tych dni to OSOBNY wiersz w arkuszu. Kolumna „Nazwa dnia”: nazwa DEFINICJI DNIA juz istniejaca w bazie enova (DefinicjeDni) - musi byc DOKLADNIE taka jak w systemie (np. „Pracy”), inaczej import zglosi blad „Definicja dnia o nazwie '' nie zostala znaleziona”. Jesli zostawisz to pole puste, uzyta zostanie wartosc domyslna z arkusza „Konfiguracja”. Kolumny Strefa 1..4: godzina rozpoczecia i czas trwania kazdej strefy tego dnia (format G:MM albo komorka sformatowana jako Godzina), np. Strefa 1 = 8:00 / 4:00, Strefa 2 = 13:00 / 4:00 (przerwa 12:00-13:00 wynika sama z luki miedzy strefami - nie wpisuje sie jej). Dzien z jedna strefa - wypelnij tylko Strefa 1, reszte zostaw pusta.</t>
   </si>
   <si>
     <t>3. W Excelu: Alt+F11 (Edytor VBA) -&gt; Plik -&gt; Importuj plik... -&gt; wskaz modGeneratorPlanuPracy.bas (w tym samym folderze co ten skoroszyt). Zapisz skoroszyt jako .xlsm (Excel z obsluga makr).</t>
@@ -72,7 +72,7 @@
     <t>Pracy</t>
   </si>
   <si>
-    <t>Nazwa definicji dnia (DefinicjeDni) w enova - domyslna nazwa systemowa dla zwyklego dnia roboczego.</t>
+    <t>Wartosc DOMYSLNA - uzywana tylko gdy w arkuszu „Plan” zostawisz puste pole „Nazwa dnia” dla danego wiersza. Musi byc nazwa definicji dnia (DefinicjeDni) juz istniejaca w bazie enova.</t>
   </si>
   <si>
     <t>Nazwa definicji strefy</t>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>Data</t>
+  </si>
+  <si>
+    <t>Nazwa dnia</t>
   </si>
   <si>
     <t>Strefa 1 od</t>
@@ -705,14 +708,15 @@
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="6" width="12.7109375" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" customWidth="1"/>
-    <col min="8" max="8" width="12.7109375" customWidth="1"/>
-    <col min="9" max="9" width="11.7109375" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.710938" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="6" max="6" width="11.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
+    <col min="10" max="10" width="11.7109375" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="7.2" customHeight="1">
@@ -746,16 +750,19 @@
       <c r="J1" s="8" t="s">
         <v>32</v>
       </c>
+      <c r="K1" s="8" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B2" s="9">
         <v>46266</v>
       </c>
       <c r="C2" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
         <v>35</v>
@@ -764,18 +771,21 @@
         <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B3" s="9">
         <v>46267</v>
       </c>
       <c r="C3" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
         <v>35</v>
@@ -784,18 +794,21 @@
         <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G3" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B4" s="9">
         <v>46268</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
         <v>35</v>
@@ -804,18 +817,21 @@
         <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B5" s="9">
         <v>46269</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
         <v>35</v>
@@ -824,18 +840,21 @@
         <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" s="9">
         <v>46270</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D6" t="s">
         <v>35</v>
@@ -844,18 +863,21 @@
         <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B7" s="9">
         <v>46271</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s">
         <v>35</v>
@@ -864,18 +886,21 @@
         <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B8" s="9">
         <v>46272</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
         <v>35</v>
@@ -884,18 +909,21 @@
         <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B9" s="9">
         <v>46273</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
         <v>35</v>
@@ -904,18 +932,21 @@
         <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10" s="9">
         <v>46274</v>
       </c>
       <c r="C10" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D10" t="s">
         <v>35</v>
@@ -924,18 +955,21 @@
         <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G10" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B11" s="9">
         <v>46275</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D11" t="s">
         <v>35</v>
@@ -944,18 +978,21 @@
         <v>36</v>
       </c>
       <c r="F11" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G11" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B12" s="9">
         <v>46276</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="D12" t="s">
         <v>35</v>
@@ -964,10 +1001,13 @@
         <v>36</v>
       </c>
       <c r="F12" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+      <c r="G12" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J12"/>
+  <autoFilter ref="A1:K12"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Generator planu pracy: dodaj kolumne Nazwa strefy (napraw definicje stref)
Drugi blad realnego testu: "Definicja strefy o nazwie 'Pracy' nie
zostala znaleziona" - Definicja strefy brana byla z globalnej
Konfiguracja, DefinicjeStref to inna lista niz DefinicjeDni. Arkusz
Plan ma teraz kolumne D "Nazwa strefy" per wiersz (fallback na
Konfiguracja!B4, blad gdy oba puste). Kolumny stref przesuniete na E..L.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AiyfQjJpMAiDQoFVsuEyaK
</commit_message>
<xml_diff>
--- a/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
+++ b/ImportyXML/Generator planu pracy/Generator planu pracy.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Plan" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Plan!$A$1:$K$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Plan!$A$1:$L$12</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -33,7 +33,7 @@
     <t>1. Arkusz „Konfiguracja”: pole „Folder na plik XML” zostaw PUSTE (plik zapisze sie obok tego skoroszytu) - chyba ze chcesz wskazac inny, JUZ ISTNIEJACY na Twoim komputerze folder. Nazwy definicji dnia/strefy zmien tylko jesli w Twojej bazie enova roznia sie od domyslnych „Pracy” / „Praca w normie”.</t>
   </si>
   <si>
-    <t>2. Uzupelnij arkusz „Plan” - jeden wiersz = jeden dzien dla jednego pracownika (Kod pracownika - dokladnie taki jak w kartotece enova - oraz Data tego konkretnego dnia). Zadnego zakresu dat ani zaznaczania dni tygodnia - jesli pracownik ma pracowac np. caly wrzesien od poniedzialku do piatku, kazdy z tych dni to OSOBNY wiersz w arkuszu. Kolumna „Nazwa dnia”: nazwa DEFINICJI DNIA juz istniejaca w bazie enova (DefinicjeDni) - musi byc DOKLADNIE taka jak w systemie (np. „Pracy”), inaczej import zglosi blad „Definicja dnia o nazwie '' nie zostala znaleziona”. Jesli zostawisz to pole puste, uzyta zostanie wartosc domyslna z arkusza „Konfiguracja”. Kolumny Strefa 1..4: godzina rozpoczecia i czas trwania kazdej strefy tego dnia (format G:MM albo komorka sformatowana jako Godzina), np. Strefa 1 = 8:00 / 4:00, Strefa 2 = 13:00 / 4:00 (przerwa 12:00-13:00 wynika sama z luki miedzy strefami - nie wpisuje sie jej). Dzien z jedna strefa - wypelnij tylko Strefa 1, reszte zostaw pusta.</t>
+    <t>2. Uzupelnij arkusz „Plan” - jeden wiersz = jeden dzien dla jednego pracownika (Kod pracownika - dokladnie taki jak w kartotece enova - oraz Data tego konkretnego dnia). Zadnego zakresu dat ani zaznaczania dni tygodnia - jesli pracownik ma pracowac np. caly wrzesien od poniedzialku do piatku, kazdy z tych dni to OSOBNY wiersz w arkuszu. Kolumna „Nazwa dnia”: nazwa DEFINICJI DNIA juz istniejaca w bazie enova (DefinicjeDni) - musi byc DOKLADNIE taka jak w systemie (np. „Pracy”), inaczej import zglosi blad „Definicja dnia o nazwie '' nie zostala znaleziona”. Kolumna „Nazwa strefy”: nazwa DEFINICJI STREFY juz istniejaca w bazie enova (DefinicjeStref - to INNA lista niz DefinicjeDni, mimo podobnych nazw!), np. „Praca w normie” - ta sama nazwa jest uzywana dla wszystkich stref 1-4 w danym wierszu. Oba pola „Nazwa dnia”/„Nazwa strefy” - jesli zostawisz puste, uzyta zostanie wartosc domyslna z arkusza „Konfiguracja”. Kolumny Strefa 1..4: godzina rozpoczecia i czas trwania kazdej strefy tego dnia (format G:MM albo komorka sformatowana jako Godzina), np. Strefa 1 = 8:00 / 4:00, Strefa 2 = 13:00 / 4:00 (przerwa 12:00-13:00 wynika sama z luki miedzy strefami - nie wpisuje sie jej). Dzien z jedna strefa - wypelnij tylko Strefa 1, reszte zostaw pusta.</t>
   </si>
   <si>
     <t>3. W Excelu: Alt+F11 (Edytor VBA) -&gt; Plik -&gt; Importuj plik... -&gt; wskaz modGeneratorPlanuPracy.bas (w tym samym folderze co ten skoroszyt). Zapisz skoroszyt jako .xlsm (Excel z obsluga makr).</t>
@@ -81,7 +81,7 @@
     <t>Praca w normie</t>
   </si>
   <si>
-    <t>Nazwa definicji strefy (DefinicjeStref) w enova - domyslna nazwa systemowa strefy pracy.</t>
+    <t>Wartosc DOMYSLNA - uzywana tylko gdy w arkuszu „Plan” zostawisz puste pole „Nazwa strefy” dla danego wiersza. Musi byc nazwa definicji strefy (DefinicjeStref - INNA lista niz DefinicjeDni) juz istniejaca w bazie enova.</t>
   </si>
   <si>
     <t>Prefiks nazwy pliku wynikowego</t>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t>Nazwa dnia</t>
+  </si>
+  <si>
+    <t>Nazwa strefy</t>
   </si>
   <si>
     <t>Strefa 1 od</t>
@@ -709,14 +712,15 @@
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" customWidth="1"/>
     <col min="3" max="3" width="16.710938" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="12.7109375" customWidth="1"/>
-    <col min="10" max="10" width="11.7109375" customWidth="1"/>
-    <col min="11" max="11" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.710938" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
+    <col min="7" max="7" width="11.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="7.2" customHeight="1">
@@ -753,10 +757,13 @@
       <c r="K1" s="8" t="s">
         <v>33</v>
       </c>
+      <c r="L1" s="8" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" s="9">
         <v>46266</v>
@@ -765,7 +772,7 @@
         <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
         <v>36</v>
@@ -774,12 +781,15 @@
         <v>37</v>
       </c>
       <c r="G2" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B3" s="9">
         <v>46267</v>
@@ -788,7 +798,7 @@
         <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
         <v>36</v>
@@ -797,12 +807,15 @@
         <v>37</v>
       </c>
       <c r="G3" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B4" s="9">
         <v>46268</v>
@@ -811,7 +824,7 @@
         <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E4" t="s">
         <v>36</v>
@@ -820,12 +833,15 @@
         <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H4" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B5" s="9">
         <v>46269</v>
@@ -834,7 +850,7 @@
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E5" t="s">
         <v>36</v>
@@ -843,12 +859,15 @@
         <v>37</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="9">
         <v>46270</v>
@@ -857,7 +876,7 @@
         <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E6" t="s">
         <v>36</v>
@@ -866,12 +885,15 @@
         <v>37</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B7" s="9">
         <v>46271</v>
@@ -880,7 +902,7 @@
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E7" t="s">
         <v>36</v>
@@ -889,12 +911,15 @@
         <v>37</v>
       </c>
       <c r="G7" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H7" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B8" s="9">
         <v>46272</v>
@@ -903,7 +928,7 @@
         <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
         <v>36</v>
@@ -912,12 +937,15 @@
         <v>37</v>
       </c>
       <c r="G8" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H8" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B9" s="9">
         <v>46273</v>
@@ -926,7 +954,7 @@
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E9" t="s">
         <v>36</v>
@@ -935,12 +963,15 @@
         <v>37</v>
       </c>
       <c r="G9" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H9" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="9">
         <v>46274</v>
@@ -949,7 +980,7 @@
         <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E10" t="s">
         <v>36</v>
@@ -958,12 +989,15 @@
         <v>37</v>
       </c>
       <c r="G10" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H10" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B11" s="9">
         <v>46275</v>
@@ -972,7 +1006,7 @@
         <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E11" t="s">
         <v>36</v>
@@ -981,12 +1015,15 @@
         <v>37</v>
       </c>
       <c r="G11" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H11" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B12" s="9">
         <v>46276</v>
@@ -995,7 +1032,7 @@
         <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="E12" t="s">
         <v>36</v>
@@ -1004,10 +1041,13 @@
         <v>37</v>
       </c>
       <c r="G12" t="s">
-        <v>36</v>
+        <v>38</v>
+      </c>
+      <c r="H12" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K12"/>
+  <autoFilter ref="A1:L12"/>
 </worksheet>
 </file>
</xml_diff>